<commit_message>
fixed minor bugs for uploading
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/STAFFS-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/STAFFS-UPLOAD-TEMPLATE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\jfdimaculangan\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\jfdimaculangan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3CCEA83-3A51-4C3B-8718-C50FF16DB6CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB722ABA-1CCB-4AE4-9F31-143E9012197B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Middle Name</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Vendor</t>
   </si>
   <si>
-    <t>Assign Status</t>
-  </si>
-  <si>
     <t>Store Request</t>
   </si>
   <si>
@@ -99,9 +96,6 @@
     <t>VENDOR 5</t>
   </si>
   <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
     <t>STORE SPECIALIST</t>
   </si>
   <si>
@@ -117,10 +111,34 @@
     <t>12312312-1231235</t>
   </si>
   <si>
-    <t>DOE 33</t>
-  </si>
-  <si>
     <t>*Date should be formatted as d/m/y</t>
+  </si>
+  <si>
+    <t>Staff Code</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>Category Type</t>
+  </si>
+  <si>
+    <t>Allowance</t>
+  </si>
+  <si>
+    <t>Salary Rate</t>
+  </si>
+  <si>
+    <t>INVENTORY AUDIT</t>
+  </si>
+  <si>
+    <t>CHOOKS TO GO</t>
+  </si>
+  <si>
+    <t>STORE REQUEST</t>
+  </si>
+  <si>
+    <t>DOE 5</t>
   </si>
 </sst>
 </file>
@@ -191,12 +209,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -512,116 +529,127 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="50.42578125" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" customWidth="1"/>
-    <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="29.85546875" customWidth="1"/>
-    <col min="10" max="10" width="49.85546875" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="39.42578125" customWidth="1"/>
-    <col min="13" max="13" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="55.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="50.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" customWidth="1"/>
+    <col min="8" max="8" width="25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="13" width="29.28515625" customWidth="1"/>
+    <col min="14" max="14" width="49.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="39.42578125" customWidth="1"/>
+    <col min="17" max="17" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="23" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="22.28515625" customWidth="1"/>
+    <col min="26" max="26" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="V1" s="2" t="s">
-        <v>22</v>
-      </c>
     </row>
-    <row r="2" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>26</v>
-      </c>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2">
         <v>9222222</v>
       </c>
-      <c r="E2" s="3">
+      <c r="F2" s="3">
         <v>46338</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
       </c>
       <c r="G2" t="s">
         <v>25</v>
@@ -630,28 +658,28 @@
         <v>23</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="L2" t="s">
-        <v>28</v>
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2">
+        <v>5312</v>
+      </c>
+      <c r="L2">
+        <v>5221</v>
       </c>
       <c r="M2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" s="3">
-        <v>46170</v>
-      </c>
-      <c r="P2" s="3">
-        <v>46170</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>46170</v>
-      </c>
-      <c r="R2" s="3">
-        <v>46170</v>
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>27</v>
       </c>
       <c r="S2" s="3">
         <v>46170</v>
@@ -662,25 +690,26 @@
       <c r="U2" s="3">
         <v>46170</v>
       </c>
+      <c r="V2" s="3">
+        <v>46170</v>
+      </c>
+      <c r="W2" s="3">
+        <v>46170</v>
+      </c>
+      <c r="X2" s="3">
+        <v>46170</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>46170</v>
+      </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="4" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>